<commit_message>
(feat) Messaging Refinement on Initial Tooling Creation
</commit_message>
<xml_diff>
--- a/assessment/self-assessment.xlsx
+++ b/assessment/self-assessment.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Individual Assessment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Team Aggregation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Assessment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Perspectives" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Framework Reference" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -546,7 +546,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Individual Assessment'!E5</f>
+              <f>'Assessment'!E5</f>
             </strRef>
           </tx>
           <spPr>
@@ -564,12 +564,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Individual Assessment'!$C$6:$C$13</f>
+              <f>'Assessment'!$C$6:$C$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Individual Assessment'!$E$6:$E$13</f>
+              <f>'Assessment'!$E$6:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -622,7 +622,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Team Automation Archetype Radar</a:t>
+              <a:t>Assessment Perspectives Radar</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -636,7 +636,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!D4</f>
+              <f>'Perspectives'!D4</f>
             </strRef>
           </tx>
           <spPr>
@@ -654,12 +654,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$D$5:$D$12</f>
+              <f>'Perspectives'!$D$5:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -668,7 +668,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!E4</f>
+              <f>'Perspectives'!E4</f>
             </strRef>
           </tx>
           <spPr>
@@ -686,12 +686,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$E$5:$E$12</f>
+              <f>'Perspectives'!$E$5:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -700,7 +700,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!F4</f>
+              <f>'Perspectives'!F4</f>
             </strRef>
           </tx>
           <spPr>
@@ -718,12 +718,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$F$5:$F$12</f>
+              <f>'Perspectives'!$F$5:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -732,7 +732,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!G4</f>
+              <f>'Perspectives'!G4</f>
             </strRef>
           </tx>
           <spPr>
@@ -750,12 +750,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$G$5:$G$12</f>
+              <f>'Perspectives'!$G$5:$G$12</f>
             </numRef>
           </val>
         </ser>
@@ -764,7 +764,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!H4</f>
+              <f>'Perspectives'!H4</f>
             </strRef>
           </tx>
           <spPr>
@@ -782,12 +782,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$H$5:$H$12</f>
+              <f>'Perspectives'!$H$5:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -796,7 +796,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!I4</f>
+              <f>'Perspectives'!I4</f>
             </strRef>
           </tx>
           <spPr>
@@ -814,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$I$5:$I$12</f>
+              <f>'Perspectives'!$I$5:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -828,7 +828,7 @@
           <order val="6"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!J4</f>
+              <f>'Perspectives'!J4</f>
             </strRef>
           </tx>
           <spPr>
@@ -846,12 +846,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$J$5:$J$12</f>
+              <f>'Perspectives'!$J$5:$J$12</f>
             </numRef>
           </val>
         </ser>
@@ -860,7 +860,7 @@
           <order val="7"/>
           <tx>
             <strRef>
-              <f>'Team Aggregation'!K4</f>
+              <f>'Perspectives'!K4</f>
             </strRef>
           </tx>
           <spPr>
@@ -878,12 +878,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Team Aggregation'!$C$5:$C$12</f>
+              <f>'Perspectives'!$C$5:$C$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Team Aggregation'!$K$5:$K$12</f>
+              <f>'Perspectives'!$K$5:$K$12</f>
             </numRef>
           </val>
         </ser>
@@ -1266,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D42"/>
+  <dimension ref="B2:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>⚙  Archetypes of Automation — Self-Assessment Workbook</t>
+          <t>Archetypes of Automation — Team Capability Assessment Workbook</t>
         </is>
       </c>
     </row>
@@ -1299,14 +1299,14 @@
     <row r="6" ht="15" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>This workbook supports the Archetypes of Automation framework — a self-assessment tool that helps individuals and teams identify strengths and gaps across 8 dimensions of automation capability.</t>
+          <t>This workbook supports the Archetypes of Automation framework — a team capability assessment tool for MSP/ITSP leaders. It is designed to be completed by a key team member or person in a position of authority evaluating their team's collective strengths and gaps.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The biggest barrier to automation in small MSP teams is not technical skill — it is process thinking, team composition, and role awareness.</t>
+          <t>The biggest barrier to automation in small MSP teams is not technical skill — it is process thinking, team composition, and role awareness. This tool helps you see where your team stands across 8 automation capability dimensions.</t>
         </is>
       </c>
     </row>
@@ -1320,49 +1320,49 @@
     <row r="10" ht="16" customHeight="1">
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Individual Assessment  →  Score yourself 0–10 per archetype. Your radar chart updates automatically.</t>
+          <t>Assessment  →  Score your team 0-10 per archetype. The radar chart updates automatically.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Team Aggregation       →  Enter each team member's scores to see the combined radar and gap analysis.</t>
+          <t>Perspectives  →  Collect assessments from multiple evaluators and compare on a shared radar.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Framework Reference    →  Full sub-archetype list with descriptions and framework citations.</t>
+          <t>Framework Reference  →  Full sub-archetype list with descriptions and framework citations.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>How to complete the Individual Assessment</t>
+          <t>How to complete the Assessment</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>1. Go to the 'Individual Assessment' sheet.</t>
+          <t>1. Go to the 'Assessment' sheet.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>2. Enter your name in the yellow Name cell (row 4).</t>
+          <t>2. Enter your name and role in the yellow Name cell (row 4).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>3. For each of the 8 archetypes, enter a score from 0–10 in the Score column.</t>
+          <t>3. For each of the 8 archetypes, enter a score from 0-10 in the Score column.</t>
         </is>
       </c>
     </row>
@@ -1376,172 +1376,186 @@
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>4. Read the sub-archetype descriptions in the 'Framework Reference' sheet to calibrate your score.</t>
+          <t>4. You are scoring your TEAM's capability, not your own personal skills.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>5. Your radar chart will update automatically as you enter scores.</t>
+          <t xml:space="preserve">   Ask yourself: does our team have someone who reliably fills this role?</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>6. Your total and profile are shown below the score table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="3" t="inlineStr">
+          <t>5. Read the sub-archetype descriptions in the 'Framework Reference' sheet to calibrate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>6. The radar chart and team profile update automatically as you enter scores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Scoring Bands</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0–2: No awareness or capability; this lens is absent</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3–4: Emerging — some instinct but no structured practice</t>
+          <t xml:space="preserve">  0-2: No one on the team fills this role; this capability is absent</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5–6: Functional — can contribute meaningfully with some gaps</t>
+          <t xml:space="preserve">  3-4: Emerging - someone shows instinct but no consistent, structured practice</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  7–8: Strong — reliable, practiced, others lean on you here</t>
+          <t xml:space="preserve">  5-6: Functional - team has some coverage here, but with notable gaps</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  9–10: Exceptional — this is a defining strength; you set the standard</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Individual Score Profiles (Total out of 80)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0–20  →  Automation Newcomer</t>
+          <t xml:space="preserve">  7-8: Strong - reliable team capability; people know who to go to</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  9-10: Exceptional - a clear team strength; this is where you set the standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Team Capability Profiles (Total out of 80)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  21–35  →  Developing Contributor</t>
+          <t xml:space="preserve">  0-20  -&gt;  Early-Stage Team</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  36–50  →  Capable Generalist</t>
+          <t xml:space="preserve">  21-35  -&gt;  Developing Team</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  51–65  →  Strong Practitioner</t>
+          <t xml:space="preserve">  36-50  -&gt;  Capable Team</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  66–80  →  Automation All-Rounder</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>How to use Team Aggregation</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>1. Each person completes their individual assessment first.</t>
+          <t xml:space="preserve">  51-65  -&gt;  Strong Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  66-80  -&gt;  High-Performing Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>How to use the Perspectives sheet</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>2. Copy each person's scores into a column on the 'Team Aggregation' sheet.</t>
+          <t>1. Have multiple evaluators (e.g. owner, ops lead, senior tech) each complete an Assessment.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>3. The combined radar chart and gap analysis update automatically.</t>
+          <t>2. Copy each evaluator's 8 scores into a column on the 'Perspectives' sheet.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>4. Look for coverage, not duplication — two 9s in Building with zero in Quality is a risk profile.</t>
+          <t>3. The combined radar chart and gap analysis update automatically.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>5. The archetype with the lowest combined average score = most urgent investment area.</t>
+          <t>4. Where perspectives diverge significantly, that disagreement is worth discussing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>5. Where all evaluators score an archetype low, that is your most urgent gap to address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>6. Use gaps to guide hiring, training, or partnership decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="37">
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B37:D37"/>
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B30:D30"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B35:D35"/>
@@ -1551,9 +1565,11 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:D43"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="B2:D2"/>
@@ -1584,19 +1600,19 @@
     <row r="1" ht="32" customHeight="1">
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>Archetypes of Automation — Individual Self-Assessment</t>
+          <t>Archetypes of Automation — Team Capability Assessment</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Name:</t>
+          <t>Name &amp; Role:</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>← Enter your name here</t>
+          <t>e.g. Jane Smith, Operations Lead</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1662,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="14">
-        <f>IF(E6&lt;=2,"0–2: No awareness; this lens is absent",IF(E6&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E6&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E6&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E6&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E6&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E6&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E6&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1668,7 +1684,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="17">
-        <f>IF(E7&lt;=2,"0–2: No awareness; this lens is absent",IF(E7&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E7&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E7&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E7&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E7&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E7&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E7&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1690,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="14">
-        <f>IF(E8&lt;=2,"0–2: No awareness; this lens is absent",IF(E8&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E8&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E8&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E8&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E8&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E8&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E8&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1712,7 +1728,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="17">
-        <f>IF(E9&lt;=2,"0–2: No awareness; this lens is absent",IF(E9&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E9&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E9&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E9&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E9&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E9&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E9&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1734,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="14">
-        <f>IF(E10&lt;=2,"0–2: No awareness; this lens is absent",IF(E10&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E10&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E10&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E10&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E10&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E10&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E10&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1756,7 +1772,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="17">
-        <f>IF(E11&lt;=2,"0–2: No awareness; this lens is absent",IF(E11&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E11&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E11&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E11&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E11&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E11&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E11&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1794,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="14">
-        <f>IF(E12&lt;=2,"0–2: No awareness; this lens is absent",IF(E12&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E12&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E12&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E12&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E12&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E12&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E12&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1800,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="17">
-        <f>IF(E13&lt;=2,"0–2: No awareness; this lens is absent",IF(E13&lt;=4,"3–4: Emerging — some instinct, no structured practice",IF(E13&lt;=6,"5–6: Functional — can contribute with some gaps",IF(E13&lt;=8,"7–8: Strong — reliable; others lean on you here","9–10: Exceptional — this is a defining strength"))))</f>
+        <f>IF(E13&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E13&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E13&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E13&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
     </row>
@@ -1818,11 +1834,11 @@
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Team Profile</t>
         </is>
       </c>
       <c r="E16" s="21">
-        <f>IF(E15&lt;=20,"Automation Newcomer",IF(E15&lt;=35,"Developing Contributor",IF(E15&lt;=50,"Capable Generalist",IF(E15&lt;=65,"Strong Practitioner","Automation All-Rounder"))))</f>
+        <f>IF(E15&lt;=20,"Early-Stage Team",IF(E15&lt;=35,"Developing Team",IF(E15&lt;=50,"Capable Team",IF(E15&lt;=65,"Strong Team","High-Performing Team"))))</f>
         <v/>
       </c>
       <c r="F16" s="22" t="n"/>
@@ -1886,56 +1902,56 @@
     <row r="1" ht="32" customHeight="1">
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>Archetypes of Automation — Team Aggregation</t>
+          <t>Archetypes of Automation — Assessment Perspectives</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>Enter each team member's scores below. The radar chart and gap analysis update automatically.</t>
+          <t>Each column = one evaluator's assessment of the team. The radar chart and gap analysis update automatically.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>Member 1 →</t>
+          <t>Evaluator 1 -&gt;</t>
         </is>
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Member 2 →</t>
+          <t>Evaluator 2 -&gt;</t>
         </is>
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
-          <t>Member 3 →</t>
+          <t>Evaluator 3 -&gt;</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
         <is>
-          <t>Member 4 →</t>
+          <t>Evaluator 4 -&gt;</t>
         </is>
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
-          <t>Member 5 →</t>
+          <t>Evaluator 5 -&gt;</t>
         </is>
       </c>
       <c r="I3" s="24" t="inlineStr">
         <is>
-          <t>Member 6 →</t>
+          <t>Evaluator 6 -&gt;</t>
         </is>
       </c>
       <c r="J3" s="24" t="inlineStr">
         <is>
-          <t>Member 7 →</t>
+          <t>Evaluator 7 -&gt;</t>
         </is>
       </c>
       <c r="K3" s="24" t="inlineStr">
         <is>
-          <t>Member 8 →</t>
+          <t>Evaluator 8 -&gt;</t>
         </is>
       </c>
     </row>
@@ -1952,42 +1968,42 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Member 1</t>
+          <t>Evaluator 1</t>
         </is>
       </c>
       <c r="E4" s="26" t="inlineStr">
         <is>
-          <t>Member 2</t>
+          <t>Evaluator 2</t>
         </is>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Member 3</t>
+          <t>Evaluator 3</t>
         </is>
       </c>
       <c r="G4" s="26" t="inlineStr">
         <is>
-          <t>Member 4</t>
+          <t>Evaluator 4</t>
         </is>
       </c>
       <c r="H4" s="25" t="inlineStr">
         <is>
-          <t>Member 5</t>
+          <t>Evaluator 5</t>
         </is>
       </c>
       <c r="I4" s="26" t="inlineStr">
         <is>
-          <t>Member 6</t>
+          <t>Evaluator 6</t>
         </is>
       </c>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>Member 7</t>
+          <t>Evaluator 7</t>
         </is>
       </c>
       <c r="K4" s="26" t="inlineStr">
         <is>
-          <t>Member 8</t>
+          <t>Evaluator 8</t>
         </is>
       </c>
       <c r="L4" s="25" t="inlineStr">

</xml_diff>